<commit_message>
feat: generate updated IPA27 analysis visualizations, datasets, documentation, and auxiliary scripts
</commit_message>
<xml_diff>
--- a/results/data/IPA27_series_finales.xlsx
+++ b/results/data/IPA27_series_finales.xlsx
@@ -472,28 +472,28 @@
         <v>42370</v>
       </c>
       <c r="B2" t="n">
-        <v>60.25</v>
+        <v>51.7</v>
       </c>
       <c r="C2" t="n">
-        <v>64.51000000000001</v>
+        <v>60.12</v>
       </c>
       <c r="D2" t="n">
-        <v>62.1</v>
+        <v>59.39</v>
       </c>
       <c r="E2" t="n">
-        <v>58.97</v>
+        <v>56.6</v>
       </c>
       <c r="F2" t="n">
-        <v>53.21</v>
+        <v>39.11</v>
       </c>
       <c r="G2" t="n">
-        <v>60.28</v>
+        <v>54.31</v>
       </c>
       <c r="H2" t="n">
-        <v>65.45</v>
+        <v>59.49</v>
       </c>
       <c r="I2" t="n">
-        <v>74.28</v>
+        <v>70.68000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -501,28 +501,28 @@
         <v>42461</v>
       </c>
       <c r="B3" t="n">
-        <v>60.06</v>
+        <v>51.71</v>
       </c>
       <c r="C3" t="n">
-        <v>64.56999999999999</v>
+        <v>60.27</v>
       </c>
       <c r="D3" t="n">
-        <v>61.92</v>
+        <v>59.42</v>
       </c>
       <c r="E3" t="n">
-        <v>58.2</v>
+        <v>55.08</v>
       </c>
       <c r="F3" t="n">
-        <v>52.89</v>
+        <v>39.22</v>
       </c>
       <c r="G3" t="n">
-        <v>61.07</v>
+        <v>56.12</v>
       </c>
       <c r="H3" t="n">
-        <v>65.36</v>
+        <v>59.32</v>
       </c>
       <c r="I3" t="n">
-        <v>74.43000000000001</v>
+        <v>70.81</v>
       </c>
     </row>
     <row r="4">
@@ -530,28 +530,28 @@
         <v>42552</v>
       </c>
       <c r="B4" t="n">
-        <v>59.37</v>
+        <v>50.72</v>
       </c>
       <c r="C4" t="n">
-        <v>64.06</v>
+        <v>59.6</v>
       </c>
       <c r="D4" t="n">
-        <v>60.25</v>
+        <v>56.91</v>
       </c>
       <c r="E4" t="n">
-        <v>57.32</v>
+        <v>53.57</v>
       </c>
       <c r="F4" t="n">
-        <v>51.89</v>
+        <v>38.29</v>
       </c>
       <c r="G4" t="n">
-        <v>60.17</v>
+        <v>55.56</v>
       </c>
       <c r="H4" t="n">
-        <v>65.97</v>
+        <v>59.87</v>
       </c>
       <c r="I4" t="n">
-        <v>74.70999999999999</v>
+        <v>71.14</v>
       </c>
     </row>
     <row r="5">
@@ -559,28 +559,28 @@
         <v>42644</v>
       </c>
       <c r="B5" t="n">
-        <v>60.07</v>
+        <v>51.57</v>
       </c>
       <c r="C5" t="n">
-        <v>64.22</v>
+        <v>59.76</v>
       </c>
       <c r="D5" t="n">
-        <v>62.13</v>
+        <v>59.2</v>
       </c>
       <c r="E5" t="n">
-        <v>57.52</v>
+        <v>53.69</v>
       </c>
       <c r="F5" t="n">
-        <v>51.85</v>
+        <v>38.55</v>
       </c>
       <c r="G5" t="n">
-        <v>60.3</v>
+        <v>55.75</v>
       </c>
       <c r="H5" t="n">
-        <v>66.22</v>
+        <v>60.08</v>
       </c>
       <c r="I5" t="n">
-        <v>74.83</v>
+        <v>71.3</v>
       </c>
     </row>
     <row r="6">
@@ -588,28 +588,28 @@
         <v>42736</v>
       </c>
       <c r="B6" t="n">
-        <v>58.8</v>
+        <v>51.11</v>
       </c>
       <c r="C6" t="n">
-        <v>64.19</v>
+        <v>60.31</v>
       </c>
       <c r="D6" t="n">
-        <v>59.05</v>
+        <v>57.77</v>
       </c>
       <c r="E6" t="n">
-        <v>56.58</v>
+        <v>53.63</v>
       </c>
       <c r="F6" t="n">
-        <v>51.3</v>
+        <v>38.43</v>
       </c>
       <c r="G6" t="n">
-        <v>60.7</v>
+        <v>57.04</v>
       </c>
       <c r="H6" t="n">
-        <v>66.05</v>
+        <v>60.12</v>
       </c>
       <c r="I6" t="n">
-        <v>75.28</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="7">
@@ -617,28 +617,28 @@
         <v>42826</v>
       </c>
       <c r="B7" t="n">
-        <v>58.73</v>
+        <v>50.8</v>
       </c>
       <c r="C7" t="n">
-        <v>63.43</v>
+        <v>59.1</v>
       </c>
       <c r="D7" t="n">
-        <v>58.51</v>
+        <v>56.96</v>
       </c>
       <c r="E7" t="n">
-        <v>54.77</v>
+        <v>51.07</v>
       </c>
       <c r="F7" t="n">
-        <v>51.32</v>
+        <v>38.07</v>
       </c>
       <c r="G7" t="n">
-        <v>60.02</v>
+        <v>56.15</v>
       </c>
       <c r="H7" t="n">
-        <v>66.36</v>
+        <v>60.46</v>
       </c>
       <c r="I7" t="n">
-        <v>75.5</v>
+        <v>71.98999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -646,28 +646,28 @@
         <v>42917</v>
       </c>
       <c r="B8" t="n">
-        <v>59.62</v>
+        <v>51.81</v>
       </c>
       <c r="C8" t="n">
-        <v>63.86</v>
+        <v>59.48</v>
       </c>
       <c r="D8" t="n">
-        <v>59.3</v>
+        <v>57.95</v>
       </c>
       <c r="E8" t="n">
-        <v>55.24</v>
+        <v>51.64</v>
       </c>
       <c r="F8" t="n">
-        <v>52.41</v>
+        <v>39.21</v>
       </c>
       <c r="G8" t="n">
-        <v>60.35</v>
+        <v>56.19</v>
       </c>
       <c r="H8" t="n">
-        <v>67.15000000000001</v>
+        <v>61.21</v>
       </c>
       <c r="I8" t="n">
-        <v>76</v>
+        <v>72.53</v>
       </c>
     </row>
     <row r="9">
@@ -675,28 +675,28 @@
         <v>43009</v>
       </c>
       <c r="B9" t="n">
-        <v>59.87</v>
+        <v>51.85</v>
       </c>
       <c r="C9" t="n">
-        <v>64.17</v>
+        <v>59.72</v>
       </c>
       <c r="D9" t="n">
-        <v>59.67</v>
+        <v>58.46</v>
       </c>
       <c r="E9" t="n">
-        <v>54.98</v>
+        <v>50.8</v>
       </c>
       <c r="F9" t="n">
-        <v>52.29</v>
+        <v>38.69</v>
       </c>
       <c r="G9" t="n">
-        <v>61.31</v>
+        <v>57.63</v>
       </c>
       <c r="H9" t="n">
-        <v>67.64</v>
+        <v>61.62</v>
       </c>
       <c r="I9" t="n">
-        <v>76.22</v>
+        <v>72.77</v>
       </c>
     </row>
     <row r="10">
@@ -704,28 +704,28 @@
         <v>43101</v>
       </c>
       <c r="B10" t="n">
-        <v>60.46</v>
+        <v>52.57</v>
       </c>
       <c r="C10" t="n">
-        <v>64.51000000000001</v>
+        <v>60.58</v>
       </c>
       <c r="D10" t="n">
-        <v>60.53</v>
+        <v>59.82</v>
       </c>
       <c r="E10" t="n">
-        <v>55.17</v>
+        <v>52.23</v>
       </c>
       <c r="F10" t="n">
-        <v>53.81</v>
+        <v>39.63</v>
       </c>
       <c r="G10" t="n">
-        <v>62.36</v>
+        <v>58.53</v>
       </c>
       <c r="H10" t="n">
-        <v>67.05</v>
+        <v>61.3</v>
       </c>
       <c r="I10" t="n">
-        <v>76.01000000000001</v>
+        <v>72.72</v>
       </c>
     </row>
     <row r="11">
@@ -733,28 +733,28 @@
         <v>43191</v>
       </c>
       <c r="B11" t="n">
-        <v>59.82</v>
+        <v>51.91</v>
       </c>
       <c r="C11" t="n">
-        <v>65.09</v>
+        <v>61.13</v>
       </c>
       <c r="D11" t="n">
-        <v>57.54</v>
+        <v>56.31</v>
       </c>
       <c r="E11" t="n">
-        <v>53.92</v>
+        <v>50.48</v>
       </c>
       <c r="F11" t="n">
-        <v>54.93</v>
+        <v>40.45</v>
       </c>
       <c r="G11" t="n">
-        <v>65.16</v>
+        <v>62</v>
       </c>
       <c r="H11" t="n">
-        <v>66.97</v>
+        <v>61.42</v>
       </c>
       <c r="I11" t="n">
-        <v>76.18000000000001</v>
+        <v>72.98</v>
       </c>
     </row>
     <row r="12">
@@ -762,28 +762,28 @@
         <v>43282</v>
       </c>
       <c r="B12" t="n">
-        <v>60.78</v>
+        <v>52.58</v>
       </c>
       <c r="C12" t="n">
-        <v>66.27</v>
+        <v>62.57</v>
       </c>
       <c r="D12" t="n">
-        <v>58.56</v>
+        <v>57.7</v>
       </c>
       <c r="E12" t="n">
-        <v>55.67</v>
+        <v>52.71</v>
       </c>
       <c r="F12" t="n">
-        <v>56.33</v>
+        <v>40.72</v>
       </c>
       <c r="G12" t="n">
-        <v>66.48</v>
+        <v>63.24</v>
       </c>
       <c r="H12" t="n">
-        <v>67.45</v>
+        <v>61.85</v>
       </c>
       <c r="I12" t="n">
-        <v>76.68000000000001</v>
+        <v>73.48</v>
       </c>
     </row>
     <row r="13">
@@ -791,28 +791,28 @@
         <v>43374</v>
       </c>
       <c r="B13" t="n">
-        <v>60.3</v>
+        <v>51.94</v>
       </c>
       <c r="C13" t="n">
-        <v>65.90000000000001</v>
+        <v>61.85</v>
       </c>
       <c r="D13" t="n">
-        <v>57.73</v>
+        <v>56.64</v>
       </c>
       <c r="E13" t="n">
-        <v>53.93</v>
+        <v>50.51</v>
       </c>
       <c r="F13" t="n">
-        <v>55.45</v>
+        <v>39.87</v>
       </c>
       <c r="G13" t="n">
-        <v>66.76000000000001</v>
+        <v>63.49</v>
       </c>
       <c r="H13" t="n">
-        <v>67.72</v>
+        <v>62.05</v>
       </c>
       <c r="I13" t="n">
-        <v>77</v>
+        <v>73.78</v>
       </c>
     </row>
     <row r="14">
@@ -820,28 +820,28 @@
         <v>43466</v>
       </c>
       <c r="B14" t="n">
-        <v>60.6</v>
+        <v>52.17</v>
       </c>
       <c r="C14" t="n">
-        <v>66.5</v>
+        <v>62.7</v>
       </c>
       <c r="D14" t="n">
-        <v>57.94</v>
+        <v>57.15</v>
       </c>
       <c r="E14" t="n">
-        <v>54.42</v>
+        <v>51.61</v>
       </c>
       <c r="F14" t="n">
-        <v>55.99</v>
+        <v>39.98</v>
       </c>
       <c r="G14" t="n">
-        <v>67.79000000000001</v>
+        <v>64.52</v>
       </c>
       <c r="H14" t="n">
-        <v>67.88</v>
+        <v>62.15</v>
       </c>
       <c r="I14" t="n">
-        <v>77.29000000000001</v>
+        <v>74.02</v>
       </c>
     </row>
     <row r="15">
@@ -849,28 +849,28 @@
         <v>43556</v>
       </c>
       <c r="B15" t="n">
-        <v>61.06</v>
+        <v>53.41</v>
       </c>
       <c r="C15" t="n">
-        <v>65.97</v>
+        <v>61.99</v>
       </c>
       <c r="D15" t="n">
-        <v>58.89</v>
+        <v>58.15</v>
       </c>
       <c r="E15" t="n">
-        <v>55.38</v>
+        <v>52.63</v>
       </c>
       <c r="F15" t="n">
-        <v>56.21</v>
+        <v>41.97</v>
       </c>
       <c r="G15" t="n">
-        <v>65</v>
+        <v>60.94</v>
       </c>
       <c r="H15" t="n">
-        <v>68.06999999999999</v>
+        <v>62.4</v>
       </c>
       <c r="I15" t="n">
-        <v>77.53</v>
+        <v>74.28</v>
       </c>
     </row>
     <row r="16">
@@ -878,28 +878,28 @@
         <v>43647</v>
       </c>
       <c r="B16" t="n">
-        <v>59.8</v>
+        <v>52.12</v>
       </c>
       <c r="C16" t="n">
-        <v>63.98</v>
+        <v>58.93</v>
       </c>
       <c r="D16" t="n">
-        <v>55.63</v>
+        <v>53.78</v>
       </c>
       <c r="E16" t="n">
-        <v>51.69</v>
+        <v>47.48</v>
       </c>
       <c r="F16" t="n">
-        <v>55.06</v>
+        <v>41.7</v>
       </c>
       <c r="G16" t="n">
-        <v>62.39</v>
+        <v>57.69</v>
       </c>
       <c r="H16" t="n">
-        <v>68.70999999999999</v>
+        <v>63.13</v>
       </c>
       <c r="I16" t="n">
-        <v>77.86</v>
+        <v>74.72</v>
       </c>
     </row>
     <row r="17">
@@ -907,28 +907,28 @@
         <v>43739</v>
       </c>
       <c r="B17" t="n">
-        <v>60.83</v>
+        <v>53.86</v>
       </c>
       <c r="C17" t="n">
-        <v>64.87</v>
+        <v>60.27</v>
       </c>
       <c r="D17" t="n">
-        <v>58.01</v>
+        <v>57.06</v>
       </c>
       <c r="E17" t="n">
-        <v>53.57</v>
+        <v>50.76</v>
       </c>
       <c r="F17" t="n">
-        <v>55.3</v>
+        <v>42.95</v>
       </c>
       <c r="G17" t="n">
-        <v>62.93</v>
+        <v>57.41</v>
       </c>
       <c r="H17" t="n">
-        <v>69.2</v>
+        <v>63.74</v>
       </c>
       <c r="I17" t="n">
-        <v>78.11</v>
+        <v>75.12</v>
       </c>
     </row>
     <row r="18">
@@ -936,28 +936,28 @@
         <v>43831</v>
       </c>
       <c r="B18" t="n">
-        <v>60.99</v>
+        <v>53.92</v>
       </c>
       <c r="C18" t="n">
-        <v>64.90000000000001</v>
+        <v>60.44</v>
       </c>
       <c r="D18" t="n">
-        <v>59.28</v>
+        <v>58.39</v>
       </c>
       <c r="E18" t="n">
-        <v>56.2</v>
+        <v>54.58</v>
       </c>
       <c r="F18" t="n">
-        <v>54.03</v>
+        <v>41.6</v>
       </c>
       <c r="G18" t="n">
-        <v>60.11</v>
+        <v>53.49</v>
       </c>
       <c r="H18" t="n">
-        <v>69.66</v>
+        <v>64.53</v>
       </c>
       <c r="I18" t="n">
-        <v>78.38</v>
+        <v>75.61</v>
       </c>
     </row>
     <row r="19">
@@ -965,28 +965,28 @@
         <v>43922</v>
       </c>
       <c r="B19" t="n">
-        <v>61.67</v>
+        <v>52.37</v>
       </c>
       <c r="C19" t="n">
-        <v>65.01000000000001</v>
+        <v>58.17</v>
       </c>
       <c r="D19" t="n">
-        <v>68.84999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>66.70999999999999</v>
+        <v>67</v>
       </c>
       <c r="F19" t="n">
-        <v>46.43</v>
+        <v>32.3</v>
       </c>
       <c r="G19" t="n">
-        <v>50.09</v>
+        <v>38.92</v>
       </c>
       <c r="H19" t="n">
-        <v>69.72</v>
+        <v>64.55</v>
       </c>
       <c r="I19" t="n">
-        <v>78.22</v>
+        <v>75.48</v>
       </c>
     </row>
     <row r="20">
@@ -994,28 +994,28 @@
         <v>44013</v>
       </c>
       <c r="B20" t="n">
-        <v>61.06</v>
+        <v>53.94</v>
       </c>
       <c r="C20" t="n">
-        <v>64.90000000000001</v>
+        <v>60.85</v>
       </c>
       <c r="D20" t="n">
-        <v>61.48</v>
+        <v>61.21</v>
       </c>
       <c r="E20" t="n">
-        <v>59.63</v>
+        <v>59.18</v>
       </c>
       <c r="F20" t="n">
-        <v>51.91</v>
+        <v>39.55</v>
       </c>
       <c r="G20" t="n">
-        <v>56.68</v>
+        <v>50.22</v>
       </c>
       <c r="H20" t="n">
-        <v>69.77</v>
+        <v>64.83</v>
       </c>
       <c r="I20" t="n">
-        <v>78.39</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="21">
@@ -1023,28 +1023,28 @@
         <v>44105</v>
       </c>
       <c r="B21" t="n">
-        <v>60.87</v>
+        <v>53.16</v>
       </c>
       <c r="C21" t="n">
-        <v>65.37</v>
+        <v>61.47</v>
       </c>
       <c r="D21" t="n">
-        <v>60.79</v>
+        <v>60.38</v>
       </c>
       <c r="E21" t="n">
-        <v>59.38</v>
+        <v>58.93</v>
       </c>
       <c r="F21" t="n">
-        <v>52.06</v>
+        <v>38.31</v>
       </c>
       <c r="G21" t="n">
-        <v>58.22</v>
+        <v>51.85</v>
       </c>
       <c r="H21" t="n">
-        <v>69.77</v>
+        <v>64.93000000000001</v>
       </c>
       <c r="I21" t="n">
-        <v>78.52</v>
+        <v>76.01000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1052,28 +1052,28 @@
         <v>44197</v>
       </c>
       <c r="B22" t="n">
-        <v>61.68</v>
+        <v>54.15</v>
       </c>
       <c r="C22" t="n">
-        <v>66.28</v>
+        <v>62.52</v>
       </c>
       <c r="D22" t="n">
-        <v>61.48</v>
+        <v>61.44</v>
       </c>
       <c r="E22" t="n">
         <v>60.19</v>
       </c>
       <c r="F22" t="n">
-        <v>53.96</v>
+        <v>39.87</v>
       </c>
       <c r="G22" t="n">
-        <v>59.79</v>
+        <v>53.18</v>
       </c>
       <c r="H22" t="n">
-        <v>69.62</v>
+        <v>64.8</v>
       </c>
       <c r="I22" t="n">
-        <v>78.87</v>
+        <v>76.34999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1081,28 +1081,28 @@
         <v>44287</v>
       </c>
       <c r="B23" t="n">
-        <v>62.26</v>
+        <v>53.46</v>
       </c>
       <c r="C23" t="n">
-        <v>66.81</v>
+        <v>63.04</v>
       </c>
       <c r="D23" t="n">
-        <v>61.33</v>
+        <v>61.35</v>
       </c>
       <c r="E23" t="n">
-        <v>59.53</v>
+        <v>59.2</v>
       </c>
       <c r="F23" t="n">
-        <v>55.76</v>
+        <v>38.38</v>
       </c>
       <c r="G23" t="n">
-        <v>61.9</v>
+        <v>55.31</v>
       </c>
       <c r="H23" t="n">
-        <v>69.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="I23" t="n">
-        <v>79</v>
+        <v>76.52</v>
       </c>
     </row>
     <row r="24">
@@ -1110,28 +1110,28 @@
         <v>44378</v>
       </c>
       <c r="B24" t="n">
-        <v>62.12</v>
+        <v>54.42</v>
       </c>
       <c r="C24" t="n">
-        <v>66.56999999999999</v>
+        <v>62.81</v>
       </c>
       <c r="D24" t="n">
-        <v>59.84</v>
+        <v>59.76</v>
       </c>
       <c r="E24" t="n">
-        <v>57.71</v>
+        <v>56.98</v>
       </c>
       <c r="F24" t="n">
-        <v>56.63</v>
+        <v>41.43</v>
       </c>
       <c r="G24" t="n">
-        <v>62.7</v>
+        <v>56.6</v>
       </c>
       <c r="H24" t="n">
-        <v>69.89</v>
+        <v>65.09</v>
       </c>
       <c r="I24" t="n">
-        <v>79.29000000000001</v>
+        <v>76.84999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1139,28 +1139,28 @@
         <v>44470</v>
       </c>
       <c r="B25" t="n">
-        <v>61.92</v>
+        <v>54.74</v>
       </c>
       <c r="C25" t="n">
-        <v>66.33</v>
+        <v>62.61</v>
       </c>
       <c r="D25" t="n">
-        <v>59.09</v>
+        <v>58.61</v>
       </c>
       <c r="E25" t="n">
-        <v>56.59</v>
+        <v>55.28</v>
       </c>
       <c r="F25" t="n">
-        <v>56.4</v>
+        <v>42.76</v>
       </c>
       <c r="G25" t="n">
-        <v>62.96</v>
+        <v>57.62</v>
       </c>
       <c r="H25" t="n">
-        <v>70.26000000000001</v>
+        <v>65.45999999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>79.45</v>
+        <v>77.04000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1168,28 +1168,28 @@
         <v>44562</v>
       </c>
       <c r="B26" t="n">
-        <v>61.85</v>
+        <v>55.97</v>
       </c>
       <c r="C26" t="n">
-        <v>65.78</v>
+        <v>61.98</v>
       </c>
       <c r="D26" t="n">
-        <v>57.81</v>
+        <v>57.04</v>
       </c>
       <c r="E26" t="n">
-        <v>55.28</v>
+        <v>53.57</v>
       </c>
       <c r="F26" t="n">
-        <v>57.03</v>
+        <v>46.64</v>
       </c>
       <c r="G26" t="n">
-        <v>62.54</v>
+        <v>57.62</v>
       </c>
       <c r="H26" t="n">
-        <v>70.69</v>
+        <v>65.91</v>
       </c>
       <c r="I26" t="n">
-        <v>79.52</v>
+        <v>77.15000000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1197,28 +1197,28 @@
         <v>44652</v>
       </c>
       <c r="B27" t="n">
-        <v>61.34</v>
+        <v>55.71</v>
       </c>
       <c r="C27" t="n">
-        <v>65.2</v>
+        <v>61.28</v>
       </c>
       <c r="D27" t="n">
-        <v>56.84</v>
+        <v>55.96</v>
       </c>
       <c r="E27" t="n">
-        <v>52.45</v>
+        <v>50.16</v>
       </c>
       <c r="F27" t="n">
-        <v>56.25</v>
+        <v>46.6</v>
       </c>
       <c r="G27" t="n">
-        <v>63.75</v>
+        <v>59.46</v>
       </c>
       <c r="H27" t="n">
-        <v>70.94</v>
+        <v>66.31999999999999</v>
       </c>
       <c r="I27" t="n">
-        <v>79.40000000000001</v>
+        <v>77.15000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1226,28 +1226,28 @@
         <v>44743</v>
       </c>
       <c r="B28" t="n">
-        <v>61.29</v>
+        <v>55.46</v>
       </c>
       <c r="C28" t="n">
-        <v>65.34</v>
+        <v>61.62</v>
       </c>
       <c r="D28" t="n">
-        <v>56.44</v>
+        <v>55.59</v>
       </c>
       <c r="E28" t="n">
-        <v>53.2</v>
+        <v>51.01</v>
       </c>
       <c r="F28" t="n">
-        <v>56.24</v>
+        <v>45.96</v>
       </c>
       <c r="G28" t="n">
-        <v>63.26</v>
+        <v>59.24</v>
       </c>
       <c r="H28" t="n">
-        <v>71.19</v>
+        <v>66.76000000000001</v>
       </c>
       <c r="I28" t="n">
-        <v>79.54000000000001</v>
+        <v>77.43000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1255,28 +1255,28 @@
         <v>44835</v>
       </c>
       <c r="B29" t="n">
-        <v>60.84</v>
+        <v>54.9</v>
       </c>
       <c r="C29" t="n">
-        <v>64.61</v>
+        <v>60.75</v>
       </c>
       <c r="D29" t="n">
-        <v>54.97</v>
+        <v>54.02</v>
       </c>
       <c r="E29" t="n">
-        <v>51.61</v>
+        <v>49.42</v>
       </c>
       <c r="F29" t="n">
-        <v>56.52</v>
+        <v>45.84</v>
       </c>
       <c r="G29" t="n">
-        <v>62.9</v>
+        <v>58.66</v>
       </c>
       <c r="H29" t="n">
-        <v>71.01000000000001</v>
+        <v>66.84</v>
       </c>
       <c r="I29" t="n">
-        <v>79.31999999999999</v>
+        <v>77.31999999999999</v>
       </c>
     </row>
     <row r="30">
@@ -1284,28 +1284,28 @@
         <v>44927</v>
       </c>
       <c r="B30" t="n">
-        <v>60.27</v>
+        <v>52.68</v>
       </c>
       <c r="C30" t="n">
-        <v>64.42</v>
+        <v>60.47</v>
       </c>
       <c r="D30" t="n">
-        <v>52.7</v>
+        <v>51.76</v>
       </c>
       <c r="E30" t="n">
-        <v>49.42</v>
+        <v>47.02</v>
       </c>
       <c r="F30" t="n">
-        <v>56.84</v>
+        <v>41.98</v>
       </c>
       <c r="G30" t="n">
-        <v>63.97</v>
+        <v>60.36</v>
       </c>
       <c r="H30" t="n">
-        <v>71.26000000000001</v>
+        <v>67.28</v>
       </c>
       <c r="I30" t="n">
-        <v>79.86</v>
+        <v>77.92</v>
       </c>
     </row>
     <row r="31">
@@ -1313,28 +1313,28 @@
         <v>45017</v>
       </c>
       <c r="B31" t="n">
-        <v>60.48</v>
+        <v>52.87</v>
       </c>
       <c r="C31" t="n">
-        <v>64.51000000000001</v>
+        <v>60.5</v>
       </c>
       <c r="D31" t="n">
-        <v>53.43</v>
+        <v>52.64</v>
       </c>
       <c r="E31" t="n">
-        <v>50.04</v>
+        <v>47.96</v>
       </c>
       <c r="F31" t="n">
-        <v>56.32</v>
+        <v>41.42</v>
       </c>
       <c r="G31" t="n">
-        <v>62.99</v>
+        <v>58.76</v>
       </c>
       <c r="H31" t="n">
-        <v>71.69</v>
+        <v>67.78</v>
       </c>
       <c r="I31" t="n">
-        <v>80.51000000000001</v>
+        <v>78.58</v>
       </c>
     </row>
     <row r="32">
@@ -1342,28 +1342,28 @@
         <v>45108</v>
       </c>
       <c r="B32" t="n">
-        <v>60.52</v>
+        <v>53.18</v>
       </c>
       <c r="C32" t="n">
-        <v>64.5</v>
+        <v>60.34</v>
       </c>
       <c r="D32" t="n">
-        <v>53.94</v>
+        <v>53.06</v>
       </c>
       <c r="E32" t="n">
-        <v>49.53</v>
+        <v>47.35</v>
       </c>
       <c r="F32" t="n">
-        <v>55.36</v>
+        <v>41.46</v>
       </c>
       <c r="G32" t="n">
-        <v>62.79</v>
+        <v>58.55</v>
       </c>
       <c r="H32" t="n">
-        <v>72.27</v>
+        <v>68.36</v>
       </c>
       <c r="I32" t="n">
-        <v>81.16</v>
+        <v>79.25</v>
       </c>
     </row>
     <row r="33">
@@ -1371,28 +1371,28 @@
         <v>45200</v>
       </c>
       <c r="B33" t="n">
-        <v>59.6</v>
+        <v>52.17</v>
       </c>
       <c r="C33" t="n">
-        <v>63.83</v>
+        <v>59.22</v>
       </c>
       <c r="D33" t="n">
-        <v>51.22</v>
+        <v>49.77</v>
       </c>
       <c r="E33" t="n">
-        <v>47.4</v>
+        <v>44.61</v>
       </c>
       <c r="F33" t="n">
-        <v>55.8</v>
+        <v>41.91</v>
       </c>
       <c r="G33" t="n">
-        <v>63.15</v>
+        <v>58.84</v>
       </c>
       <c r="H33" t="n">
-        <v>71.79000000000001</v>
+        <v>68.08</v>
       </c>
       <c r="I33" t="n">
-        <v>80.95</v>
+        <v>79.13</v>
       </c>
     </row>
     <row r="34">
@@ -1400,28 +1400,28 @@
         <v>45292</v>
       </c>
       <c r="B34" t="n">
-        <v>60.12</v>
+        <v>53.25</v>
       </c>
       <c r="C34" t="n">
-        <v>64.44</v>
+        <v>59.88</v>
       </c>
       <c r="D34" t="n">
-        <v>52.16</v>
+        <v>50.97</v>
       </c>
       <c r="E34" t="n">
-        <v>48.09</v>
+        <v>45.58</v>
       </c>
       <c r="F34" t="n">
-        <v>56.44</v>
+        <v>43.59</v>
       </c>
       <c r="G34" t="n">
-        <v>64.17</v>
+        <v>59.46</v>
       </c>
       <c r="H34" t="n">
-        <v>71.77</v>
+        <v>67.95999999999999</v>
       </c>
       <c r="I34" t="n">
-        <v>81.06</v>
+        <v>79.23</v>
       </c>
     </row>
     <row r="35">
@@ -1429,28 +1429,28 @@
         <v>45383</v>
       </c>
       <c r="B35" t="n">
-        <v>60.93</v>
+        <v>54.28</v>
       </c>
       <c r="C35" t="n">
-        <v>65.15000000000001</v>
+        <v>61.12</v>
       </c>
       <c r="D35" t="n">
-        <v>53.2</v>
+        <v>51.91</v>
       </c>
       <c r="E35" t="n">
-        <v>48.76</v>
+        <v>46.34</v>
       </c>
       <c r="F35" t="n">
-        <v>57.59</v>
+        <v>45.24</v>
       </c>
       <c r="G35" t="n">
-        <v>65.55</v>
+        <v>62.11</v>
       </c>
       <c r="H35" t="n">
-        <v>72</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="I35" t="n">
-        <v>81.15000000000001</v>
+        <v>79.31999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -1458,28 +1458,28 @@
         <v>45474</v>
       </c>
       <c r="B36" t="n">
-        <v>61.96</v>
+        <v>54.79</v>
       </c>
       <c r="C36" t="n">
-        <v>66.20999999999999</v>
+        <v>62.29</v>
       </c>
       <c r="D36" t="n">
-        <v>54.37</v>
+        <v>53.16</v>
       </c>
       <c r="E36" t="n">
-        <v>50.29</v>
+        <v>48.13</v>
       </c>
       <c r="F36" t="n">
-        <v>58.91</v>
+        <v>45.15</v>
       </c>
       <c r="G36" t="n">
-        <v>66.69</v>
+        <v>62.94</v>
       </c>
       <c r="H36" t="n">
-        <v>72.59999999999999</v>
+        <v>68.53</v>
       </c>
       <c r="I36" t="n">
-        <v>81.64</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="37">
@@ -1487,28 +1487,28 @@
         <v>45566</v>
       </c>
       <c r="B37" t="n">
-        <v>61.82</v>
+        <v>55.06</v>
       </c>
       <c r="C37" t="n">
-        <v>66.12</v>
+        <v>61.94</v>
       </c>
       <c r="D37" t="n">
-        <v>53.77</v>
+        <v>51.89</v>
       </c>
       <c r="E37" t="n">
-        <v>48.98</v>
+        <v>46.41</v>
       </c>
       <c r="F37" t="n">
-        <v>59.76</v>
+        <v>47.34</v>
       </c>
       <c r="G37" t="n">
-        <v>67.93000000000001</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="H37" t="n">
-        <v>71.92</v>
+        <v>67.97</v>
       </c>
       <c r="I37" t="n">
-        <v>81.44</v>
+        <v>79.64</v>
       </c>
     </row>
     <row r="38">
@@ -1516,28 +1516,28 @@
         <v>45658</v>
       </c>
       <c r="B38" t="n">
-        <v>61.99</v>
+        <v>55.06</v>
       </c>
       <c r="C38" t="n">
-        <v>65.69</v>
+        <v>61.41</v>
       </c>
       <c r="D38" t="n">
-        <v>55</v>
+        <v>53.14</v>
       </c>
       <c r="E38" t="n">
-        <v>49.19</v>
+        <v>46.69</v>
       </c>
       <c r="F38" t="n">
-        <v>59.06</v>
+        <v>46.29</v>
       </c>
       <c r="G38" t="n">
-        <v>66.41</v>
+        <v>62.23</v>
       </c>
       <c r="H38" t="n">
-        <v>71.91</v>
+        <v>67.87</v>
       </c>
       <c r="I38" t="n">
-        <v>81.48</v>
+        <v>79.69</v>
       </c>
     </row>
     <row r="39">
@@ -1545,28 +1545,28 @@
         <v>45748</v>
       </c>
       <c r="B39" t="n">
-        <v>62.51</v>
+        <v>55.54</v>
       </c>
       <c r="C39" t="n">
-        <v>65.87</v>
+        <v>61.15</v>
       </c>
       <c r="D39" t="n">
-        <v>54.85</v>
+        <v>52.71</v>
       </c>
       <c r="E39" t="n">
-        <v>48.77</v>
+        <v>46.14</v>
       </c>
       <c r="F39" t="n">
-        <v>60.55</v>
+        <v>47.73</v>
       </c>
       <c r="G39" t="n">
-        <v>67.31999999999999</v>
+        <v>62.14</v>
       </c>
       <c r="H39" t="n">
-        <v>72.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="I39" t="n">
-        <v>81.52</v>
+        <v>79.76000000000001</v>
       </c>
     </row>
     <row r="40">
@@ -1574,28 +1574,28 @@
         <v>45839</v>
       </c>
       <c r="B40" t="n">
-        <v>62.87</v>
+        <v>56.61</v>
       </c>
       <c r="C40" t="n">
-        <v>65.88</v>
+        <v>60.84</v>
       </c>
       <c r="D40" t="n">
-        <v>54.71</v>
+        <v>52.24</v>
       </c>
       <c r="E40" t="n">
-        <v>47.74</v>
+        <v>44.14</v>
       </c>
       <c r="F40" t="n">
-        <v>61.39</v>
+        <v>50.67</v>
       </c>
       <c r="G40" t="n">
-        <v>68.37</v>
+        <v>63.91</v>
       </c>
       <c r="H40" t="n">
-        <v>72.51000000000001</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="I40" t="n">
-        <v>81.53</v>
+        <v>79.81999999999999</v>
       </c>
     </row>
     <row r="41">
@@ -1603,28 +1603,28 @@
         <v>45931</v>
       </c>
       <c r="B41" t="n">
-        <v>63.26</v>
+        <v>56.97</v>
       </c>
       <c r="C41" t="n">
-        <v>66.20999999999999</v>
+        <v>61.6</v>
       </c>
       <c r="D41" t="n">
-        <v>55.4</v>
+        <v>53.28</v>
       </c>
       <c r="E41" t="n">
-        <v>48.46</v>
+        <v>45.88</v>
       </c>
       <c r="F41" t="n">
-        <v>61.99</v>
+        <v>50.65</v>
       </c>
       <c r="G41" t="n">
-        <v>68.41</v>
+        <v>63.66</v>
       </c>
       <c r="H41" t="n">
-        <v>72.38</v>
+        <v>68.48999999999999</v>
       </c>
       <c r="I41" t="n">
-        <v>81.75</v>
+        <v>80.05</v>
       </c>
     </row>
     <row r="42">
@@ -1632,28 +1632,28 @@
         <v>46023</v>
       </c>
       <c r="B42" t="n">
-        <v>63.84</v>
+        <v>57.54</v>
       </c>
       <c r="C42" t="n">
-        <v>66.59</v>
+        <v>62.23</v>
       </c>
       <c r="D42" t="n">
-        <v>56.54</v>
+        <v>54.77</v>
       </c>
       <c r="E42" t="n">
-        <v>49.08</v>
+        <v>46.65</v>
       </c>
       <c r="F42" t="n">
-        <v>62.2</v>
+        <v>50.47</v>
       </c>
       <c r="G42" t="n">
-        <v>68.76000000000001</v>
+        <v>64.38</v>
       </c>
       <c r="H42" t="n">
-        <v>72.78</v>
+        <v>68.92</v>
       </c>
       <c r="I42" t="n">
-        <v>81.92</v>
+        <v>80.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>